<commit_message>
Add Ubuntu GUI build, K1V2SPI User Guides, firmware rename; move docs to Private
GUI
- Cross-platform GUI: fonts, settings dir (~/.config on Linux), xdg-open, serial port hint
- Build outputs per OS: gui/Win (build_win.bat, dist/*.exe) and gui/Linux
  (build_linux.sh, build_linux_docker.bat, dist/K1V2SPI_Programmer for Ubuntu 22.04+)
- gui/Win/build and gui/Linux/build are PyInstaller work files: now git-ignored

Firmware
- Prebuilt HEX renamed to K1V2SPI_FW_PIC18F16Q20.hex (build.bat, flash_nano.bat updated)

Docs
- User Manual/: K1V2SPI Programmer User Guide (Traditional Chinese, English)
- README, ChangeHistory and docs/ now live in the private repo (Private/); BD, Datasheet,
  tests and tools are in Private/ as well. build_win.bat and flash_nano.bat call
  Private/tools/py.cmd

Hardware
- Add BOM export (Project_Outputs), block diagram, schematic PDF, OutJob and BomDoc

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hardware/BOM_Template.xlsx
+++ b/Hardware/BOM_Template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5CB0EE-9182-4173-8B6C-A9F6B542FB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{AB5CB0EE-9182-4173-8B6C-A9F6B542FB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CCB4375-A80A-44D9-BE2E-B25132C78117}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part List Report" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Part List Report'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Part List Report'!$A$1:$I$38</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,13 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
-  <si>
-    <t>Field=VariantName</t>
-  </si>
-  <si>
-    <t>Field=TotalQuantity</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="120">
   <si>
     <t>Variant:</t>
   </si>
@@ -47,9 +41,6 @@
     <t>Component list</t>
   </si>
   <si>
-    <t>Column=Quantity</t>
-  </si>
-  <si>
     <t>Approved</t>
   </si>
   <si>
@@ -59,43 +50,346 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>Column=Designator</t>
-  </si>
-  <si>
-    <t>Column=Value</t>
-  </si>
-  <si>
-    <t>Field=CurrentDate</t>
-  </si>
-  <si>
-    <t>Field=CurrentTime</t>
-  </si>
-  <si>
-    <t>Column=Fitted</t>
-  </si>
-  <si>
-    <t>Column=Manufacturer 1</t>
-  </si>
-  <si>
-    <t>Column=Manufacturer Part Number 1</t>
-  </si>
-  <si>
-    <t>Column=Description_</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Field=ProjectTitle </t>
-  </si>
-  <si>
-    <t>Field=ProjectPCBAssyNumber</t>
-  </si>
-  <si>
     <t>PCBA Number:</t>
   </si>
   <si>
-    <t>Field=ProjectPCBAssyRevision</t>
-  </si>
-  <si>
     <t>PCBA Revision:</t>
+  </si>
+  <si>
+    <t>PIC18F16Q20 Curiosity Nano</t>
+  </si>
+  <si>
+    <t>02-00457</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Default Assembly</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>12:19:53 AM</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>#Column Name Error:' Fitted</t>
+  </si>
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t>C1, C2, C3, C4, C5, C100, C101, C102, C103, C104, C105, C200, C201, C202, C203, C204, C206, C207, C208, C209</t>
+  </si>
+  <si>
+    <t>C205</t>
+  </si>
+  <si>
+    <t>D100</t>
+  </si>
+  <si>
+    <t>D200</t>
+  </si>
+  <si>
+    <t>J107, J108</t>
+  </si>
+  <si>
+    <t>J203</t>
+  </si>
+  <si>
+    <t>LABEL1</t>
+  </si>
+  <si>
+    <t>Q200</t>
+  </si>
+  <si>
+    <t>Q201</t>
+  </si>
+  <si>
+    <t>R1, R2, R3, R4, R5, R6, R7, R8, R9, R10, R11, R12, R13, R14, R15, R16, R17, R18, R19, R100, R101, R102, R103, R104, R105, R106, R200, R201, R202, R203, R204, R205, R206, R207, R208, R209, R210, R211, R212, R213, R214, R215, R216, R217, R218</t>
+  </si>
+  <si>
+    <t>SKT1</t>
+  </si>
+  <si>
+    <t>SW100</t>
+  </si>
+  <si>
+    <t>Test1, Test2</t>
+  </si>
+  <si>
+    <t>TEST FIXTURE1</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>U100</t>
+  </si>
+  <si>
+    <t>U101</t>
+  </si>
+  <si>
+    <t>U200</t>
+  </si>
+  <si>
+    <t>U201</t>
+  </si>
+  <si>
+    <t>U202</t>
+  </si>
+  <si>
+    <t>U203</t>
+  </si>
+  <si>
+    <t>U204, U205, U207, U208, U209</t>
+  </si>
+  <si>
+    <t>U206</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>4.7uF, 1uF, 0.1uF, 2.2uF, 2200pF</t>
+  </si>
+  <si>
+    <t>4.7uF</t>
+  </si>
+  <si>
+    <t>Yellow LED</t>
+  </si>
+  <si>
+    <t>LED SINGLE SML-P12MTT86R YELLOW-GREEN</t>
+  </si>
+  <si>
+    <t>HDR-2.54 Male 1x2</t>
+  </si>
+  <si>
+    <t>USB2.0 Type-C FEMALE</t>
+  </si>
+  <si>
+    <t>PCBA LABEL 18X6mm</t>
+  </si>
+  <si>
+    <t>DMN65D8LFB-7B</t>
+  </si>
+  <si>
+    <t>CSD25501F3</t>
+  </si>
+  <si>
+    <t>0R, 20k, 10k, 200k, 82R, 300R, 47k, 1k, 27k, 33k, 470R, 5.1k</t>
+  </si>
+  <si>
+    <t>OTS-8(16)-1.27-03</t>
+  </si>
+  <si>
+    <t>TACT SPST</t>
+  </si>
+  <si>
+    <t>[NoValue], Debugger Firmware</t>
+  </si>
+  <si>
+    <t>Curiosity Nano Test Fixture</t>
+  </si>
+  <si>
+    <t>MCP1826</t>
+  </si>
+  <si>
+    <t>PIC18F16Q20</t>
+  </si>
+  <si>
+    <t>MCP1711/1.2V</t>
+  </si>
+  <si>
+    <t>MIC5353YMT-TR</t>
+  </si>
+  <si>
+    <t>MIC94163YCS</t>
+  </si>
+  <si>
+    <t>MIC2008</t>
+  </si>
+  <si>
+    <t>MIC5528 3V3</t>
+  </si>
+  <si>
+    <t>74LVC1T45FW4-7</t>
+  </si>
+  <si>
+    <t>ATSAMD21E18</t>
+  </si>
+  <si>
+    <t>Manufacturer 1</t>
+  </si>
+  <si>
+    <t>TDK Corporation, Murata, Yageo, Hottech, KEMET</t>
+  </si>
+  <si>
+    <t>KEMET</t>
+  </si>
+  <si>
+    <t>Rohm Semiconductor</t>
+  </si>
+  <si>
+    <t>Würth Elektronik</t>
+  </si>
+  <si>
+    <t>KLS Electronic</t>
+  </si>
+  <si>
+    <t>ACT Logimark AS</t>
+  </si>
+  <si>
+    <t>Diodes Incorporated</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>Bourns, Yageo, Vishay, Panasonic, Panasonic Electronic Components</t>
+  </si>
+  <si>
+    <t>Enplas</t>
+  </si>
+  <si>
+    <t>Raynen</t>
+  </si>
+  <si>
+    <t>Microchip Technology</t>
+  </si>
+  <si>
+    <t>Manufacturer Part Number 1</t>
+  </si>
+  <si>
+    <t>C1005X5R1A475K050BC, GRM155C71C105KE11J, CC0402KRX5R6BB104, C1005B104K160NT, C1005A225K100NT, C0402C105K9PACTU, C0402C222J3GACTU</t>
+  </si>
+  <si>
+    <t>C0603C475K8PACTU</t>
+  </si>
+  <si>
+    <t>SML-D12Y1WT86</t>
+  </si>
+  <si>
+    <t>SML-P12MTT86R</t>
+  </si>
+  <si>
+    <t>L-KLS1-5409-R</t>
+  </si>
+  <si>
+    <t>DMN65D8LFB-7</t>
+  </si>
+  <si>
+    <t>CR0402-J/-000GLF, RC0402FR-0720KL, MCS0402MC1002FE000, RC0402FR-07200KL, CR0402-JW-820GLF, RC0402JR-07300RL, RC0402FR-0747KL, ERJ-2RKF1001X, RC0402JR-070RL, RC0402FR-0727KL, AC0402FR-0733KL, RC0402FR-07470RL, ERJ-2RKF5101X</t>
+  </si>
+  <si>
+    <t>L-KLS7-TS0304A-2-300-T</t>
+  </si>
+  <si>
+    <t>MCHP 15-00009</t>
+  </si>
+  <si>
+    <t>MCP1826T-1802E/DC</t>
+  </si>
+  <si>
+    <t>PIC18F16Q20T-I/REB</t>
+  </si>
+  <si>
+    <t>MCP1711T-12I/5X</t>
+  </si>
+  <si>
+    <t>MIC94163YCS-TR</t>
+  </si>
+  <si>
+    <t>MIC2008YML-TR</t>
+  </si>
+  <si>
+    <t>MIC5528-3.3YMT-TR</t>
+  </si>
+  <si>
+    <t>ATSAMD21E18A-MUT</t>
+  </si>
+  <si>
+    <t>Description_</t>
+  </si>
+  <si>
+    <t>CAP CER 4.7uF 10V 10% X5R SMD 0402, CAP CER 1uF 16V 10% X7S SMD 0402, CAP CER 0.1UF 10V ±10% X5R SMD 0402, CAP CER 0.1uF 16V 10% X7R SMD 0402, CAP CER 2.2uF 10V 10% X5R SMD 0402, CAP CER 1uF 6.3V 10% X5R SMD 0402, CAP CER 2200pF 25V 5% C0G SMD 0402</t>
+  </si>
+  <si>
+    <t>CAP CER 4.7uF 10V 10% X5R SMD 0603</t>
+  </si>
+  <si>
+    <t>LED YELLOW DIFFUSED 1608 SMD</t>
+  </si>
+  <si>
+    <t>DIO LED YELLOW-GREEN 2.2V 20mA 25mcd Clear SMD 0402</t>
+  </si>
+  <si>
+    <t>CON HDR-2.54 Male 1x2 Gold 5.84MH TH VERT</t>
+  </si>
+  <si>
+    <t>CON USB2.0 Type-C Female SMD R/A</t>
+  </si>
+  <si>
+    <t>LABEL PCBA 18x6mm Datamatrix Assy# / Rev / Serial / Date</t>
+  </si>
+  <si>
+    <t>TRANS FET N-CH DMN65D8LFB-7B 260mA 60V 430mW X1_DFN1006-3</t>
+  </si>
+  <si>
+    <t>TRANS FET P-CH CSD25501F3 -20V -3.6A 0.076R LGA</t>
+  </si>
+  <si>
+    <t>RES TKF 0R 1/16W SMD 0402, RES TKF 20K 1% 1/16W SMD 0402, RES TF 10k 1% 1/10W SMD 0402 AEC-Q200, RES TKF 200k 1% 1/16W SMD 0402, RES TKF 82R 5% 1/16W SMD 0402, RES TKF 300R 5% 1/16W SMD 0402, RES TKF 47k 1% 1/16W SMD 0402, RES TKF 1k 1% 1/10W SMD 0402, RES TKF 27k 1% 1/16W SMD 0402, RES TKF 33k 1% 1/16W SMD 0402, RES TKF 470R 1% 1/16W MF 0402, RES TKF 5.1k 1% 1/10W SMD 0402</t>
+  </si>
+  <si>
+    <t>SOCKET IC CLAMP SOP-8 SO-8</t>
+  </si>
+  <si>
+    <t>SWITCH TACT SPST 12V 50mA L-KLS7-TS0304A-2-300-T SMD</t>
+  </si>
+  <si>
+    <t>TEST, PIC18F16Q20-CNANO, FW, CNANO-DEBUGGER</t>
+  </si>
+  <si>
+    <t>MCHP ANALOG LDO 1.8V MCP1826T-1802E/DC SOT-223-5</t>
+  </si>
+  <si>
+    <t>IC VOLTAGE TRANSLATOR BI-DIR 8 CIRCUIT LSF0108PWR TSSOP20</t>
+  </si>
+  <si>
+    <t>MCHP MCU 8-BIT 64MHz 64KB 4KB PIC18F16Q20T-I/REB VQFN-20</t>
+  </si>
+  <si>
+    <t>MCHP ANALOG LDO 1.2V MCP1711T-12I/5X UQFN-4</t>
+  </si>
+  <si>
+    <t>MCHP ANALOG LDO ADJ 500mA MIC5353YMT-TR MLF-6</t>
+  </si>
+  <si>
+    <t>IC LOAD SWITCH HI SIDE 3A 6WLCSP</t>
+  </si>
+  <si>
+    <t>MCHP ANALOG POWER SWITCH 5.5V 2.1A MIC2008YML-TR VDFN-6</t>
+  </si>
+  <si>
+    <t>MCHP ANALOG LDO 3.3V MIC5528-3.3YMT-TR 6-TDFN</t>
+  </si>
+  <si>
+    <t>IC VOLTAGE TRANSLATOR BI-DIR 1 CIRCUIT 74LVC1T45FW4-7 X2-DFN1010-6</t>
+  </si>
+  <si>
+    <t>MCHP MCU 32-BIT 48MHz 256Kb 32Kb ATSAMD21E18A-MUT QFN-32</t>
   </si>
 </sst>
 </file>
@@ -529,7 +823,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -572,9 +866,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -624,9 +915,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -676,12 +964,6 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -691,16 +973,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -714,6 +987,21 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -811,7 +1099,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>5182415</xdr:colOff>
+      <xdr:colOff>5172890</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>172418</xdr:rowOff>
     </xdr:to>
@@ -1169,12 +1457,12 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" style="21" customWidth="1"/>
-    <col min="3" max="3" width="24" style="21" customWidth="1"/>
+    <col min="2" max="2" width="6.85546875" style="20" customWidth="1"/>
+    <col min="3" max="3" width="24" style="20" customWidth="1"/>
     <col min="4" max="4" width="16" style="4" customWidth="1"/>
     <col min="5" max="5" width="20.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="33.42578125" style="1" customWidth="1"/>
@@ -1185,242 +1473,751 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46"/>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="33"/>
+      <c r="A1" s="44"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="31"/>
     </row>
     <row r="2" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="47"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="26"/>
-      <c r="E2" s="62" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="34"/>
+      <c r="A2" s="45"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="25"/>
+      <c r="E2" s="60" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="32"/>
     </row>
     <row r="3" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="47"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>18</v>
+      <c r="A3" s="45"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="61" t="s">
+        <v>9</v>
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
-      <c r="I3" s="35"/>
+      <c r="I3" s="33"/>
     </row>
     <row r="4" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="47"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="64" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="63" t="s">
-        <v>20</v>
+      <c r="A4" s="45"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="57" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="56" t="s">
+        <v>10</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
-      <c r="I4" s="35"/>
+      <c r="I4" s="33"/>
     </row>
     <row r="5" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="47"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="27" t="s">
-        <v>2</v>
-      </c>
-      <c r="E5" s="63" t="s">
+      <c r="A5" s="45"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="26" t="s">
         <v>0</v>
+      </c>
+      <c r="E5" s="56" t="s">
+        <v>11</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="12"/>
       <c r="H5" s="12"/>
-      <c r="I5" s="35"/>
+      <c r="I5" s="33"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="47"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="17"/>
+      <c r="A6" s="45"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="16"/>
       <c r="D6" s="11"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="15"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="14"/>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
-      <c r="I6" s="35"/>
+      <c r="I6" s="33"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="47"/>
-      <c r="B7" s="57"/>
-      <c r="C7" s="58" t="s">
+      <c r="A7" s="45"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="54" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="63" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="55"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="33"/>
+    </row>
+    <row r="8" spans="1:9" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="45"/>
+      <c r="B8" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="49" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="49" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="49" t="s">
+        <v>79</v>
+      </c>
+      <c r="H8" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" s="34"/>
+    </row>
+    <row r="9" spans="1:9" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A9" s="45"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="50">
+        <v>20</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="50" t="s">
+        <v>80</v>
+      </c>
+      <c r="H9" s="51" t="s">
+        <v>97</v>
+      </c>
+      <c r="I9" s="35"/>
+    </row>
+    <row r="10" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="45"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="22">
+        <v>1</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="I10" s="35"/>
+    </row>
+    <row r="11" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="45"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="50">
+        <v>1</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="H11" s="51" t="s">
+        <v>99</v>
+      </c>
+      <c r="I11" s="35"/>
+    </row>
+    <row r="12" spans="1:9" s="3" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="45"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="22">
+        <v>1</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="I12" s="35"/>
+    </row>
+    <row r="13" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="45"/>
+      <c r="B13" s="50"/>
+      <c r="C13" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="50">
+        <v>2</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="50">
+        <v>61300211121</v>
+      </c>
+      <c r="H13" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="I13" s="35"/>
+    </row>
+    <row r="14" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="45"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="22">
+        <v>1</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="I14" s="35"/>
+    </row>
+    <row r="15" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="45"/>
+      <c r="B15" s="50"/>
+      <c r="C15" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="50">
+        <v>1</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="50" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" s="50">
+        <v>505462</v>
+      </c>
+      <c r="H15" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="I15" s="35"/>
+    </row>
+    <row r="16" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="45"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="22">
+        <v>1</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="H16" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="I16" s="35"/>
+    </row>
+    <row r="17" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="45"/>
+      <c r="B17" s="50"/>
+      <c r="C17" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="50">
+        <v>1</v>
+      </c>
+      <c r="E17" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="F17" s="50" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="H17" s="51" t="s">
+        <v>105</v>
+      </c>
+      <c r="I17" s="35"/>
+    </row>
+    <row r="18" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.2">
+      <c r="A18" s="45"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="22">
+        <v>45</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="I18" s="35"/>
+    </row>
+    <row r="19" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="45"/>
+      <c r="B19" s="50"/>
+      <c r="C19" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="50">
+        <v>1</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="H19" s="51" t="s">
+        <v>107</v>
+      </c>
+      <c r="I19" s="35"/>
+    </row>
+    <row r="20" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="45"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="22">
+        <v>1</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="I20" s="35"/>
+    </row>
+    <row r="21" spans="1:9" s="3" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A21" s="45"/>
+      <c r="B21" s="50"/>
+      <c r="C21" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="50">
+        <v>2</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="50"/>
+      <c r="G21" s="50"/>
+      <c r="H21" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="I21" s="35"/>
+    </row>
+    <row r="22" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="45"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="22">
+        <v>1</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="H22" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="I22" s="35"/>
+    </row>
+    <row r="23" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="45"/>
+      <c r="B23" s="50"/>
+      <c r="C23" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="50">
+        <v>1</v>
+      </c>
+      <c r="E23" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="G23" s="50" t="s">
+        <v>89</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="I23" s="35"/>
+    </row>
+    <row r="24" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="45"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="22">
+        <v>1</v>
+      </c>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="I24" s="35"/>
+    </row>
+    <row r="25" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="45"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" s="50">
+        <v>1</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>58</v>
+      </c>
+      <c r="F25" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="G25" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" s="51" t="s">
+        <v>112</v>
+      </c>
+      <c r="I25" s="35"/>
+    </row>
+    <row r="26" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="45"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="22">
+        <v>1</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="F26" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="G26" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="H26" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="I26" s="35"/>
+    </row>
+    <row r="27" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="45"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="50" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" s="50">
+        <v>1</v>
+      </c>
+      <c r="E27" s="50" t="s">
+        <v>60</v>
+      </c>
+      <c r="F27" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="G27" s="50" t="s">
+        <v>60</v>
+      </c>
+      <c r="H27" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="I27" s="35"/>
+    </row>
+    <row r="28" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="45"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28" s="22">
+        <v>1</v>
+      </c>
+      <c r="E28" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="G28" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="H28" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="I28" s="35"/>
+    </row>
+    <row r="29" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="45"/>
+      <c r="B29" s="50"/>
+      <c r="C29" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="50">
+        <v>1</v>
+      </c>
+      <c r="E29" s="50" t="s">
+        <v>62</v>
+      </c>
+      <c r="F29" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="G29" s="50" t="s">
+        <v>93</v>
+      </c>
+      <c r="H29" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="I29" s="35"/>
+    </row>
+    <row r="30" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="45"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="22">
+        <v>1</v>
+      </c>
+      <c r="E30" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="F30" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="G30" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="H30" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="I30" s="35"/>
+    </row>
+    <row r="31" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="45"/>
+      <c r="B31" s="50"/>
+      <c r="C31" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" s="50">
+        <v>5</v>
+      </c>
+      <c r="E31" s="50" t="s">
+        <v>64</v>
+      </c>
+      <c r="F31" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="G31" s="50" t="s">
+        <v>64</v>
+      </c>
+      <c r="H31" s="51" t="s">
+        <v>118</v>
+      </c>
+      <c r="I31" s="35"/>
+    </row>
+    <row r="32" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="45"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D32" s="22">
+        <v>1</v>
+      </c>
+      <c r="E32" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="F32" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="G32" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="I32" s="35"/>
+    </row>
+    <row r="33" spans="1:9" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="46"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="64" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="36"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="45"/>
+      <c r="B34" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="59" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="60" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="61"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="35"/>
-    </row>
-    <row r="8" spans="1:9" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="47"/>
-      <c r="B8" s="50" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="51" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="51" t="s">
+      <c r="C34" s="59"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="I34" s="37"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" s="45"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="38"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" s="45"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="38"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" s="45"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="51" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="51" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="51" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="51" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="36"/>
-    </row>
-    <row r="9" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="47"/>
-      <c r="B9" s="52"/>
-      <c r="C9" s="52"/>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="52"/>
-      <c r="H9" s="53"/>
-      <c r="I9" s="37"/>
-    </row>
-    <row r="10" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="47"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="37"/>
-    </row>
-    <row r="11" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="47"/>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="37"/>
-    </row>
-    <row r="12" spans="1:9" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="48"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="32" t="s">
-        <v>1</v>
-      </c>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="31"/>
-      <c r="I12" s="38"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="47"/>
-      <c r="B13" s="65" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="66"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="I13" s="39"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="47"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="40"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="47"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="40"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="47"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I16" s="40"/>
-    </row>
-    <row r="17" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="49"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="41"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="D21" s="1"/>
+      <c r="I37" s="38"/>
+    </row>
+    <row r="38" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="47"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="39"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D40" s="1"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D41" s="1"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D42" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B34:C34"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>